<commit_message>
Fix moral weights and cost assumptions in oxygen therapy analysis
Corrects three errors in the oxygen therapy BOTEC flagged by reviewer:
- Child moral weight: 52.5 -> 117 (GiveWell 2020 weights: Post Neonatal
  100.7, 1-4yr 127.3, weighted avg)
- Adult moral weight: 30 -> 100 (weighted avg across ages 20-50)
- Cost per patient: $30 "philanthropic" -> $45 total program cost,
  triangulated across CHAI ($45), Bradley 2021 ($26), Lancet Commission
  ($59/DALY)

Adds docs/moral_weights.md with the full GiveWell 2020 moral weights
table for local reference. Updates methodology.md to reference
age-specific weights instead of a single blanket number.

New bottom line: ~15x at $45/patient (was 9.8x at $30/patient).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/botecs/oxygen_therapy_for_children.xlsx
+++ b/outputs/botecs/oxygen_therapy_for_children.xlsx
@@ -171,7 +171,7 @@
   <commentList>
     <comment ref="C3" authorId="0" shapeId="0">
       <text>
-        <t>Original BOTEC used $15.12 (CHAI) + $15.12 (government) + $15.12 (additional) = $45.35 total. Using $30 as philanthropic cost (CHAI + additional, excluding government match). Malawi CEA (Lin et al. 2025) implies much lower per-patient costs at scale. This is a key assumption — sensitivity from $15 to $50.</t>
+        <t>Three independent estimates: (1) Original CHAI BOTEC: $15.12 CHAI + $15.12 govt + $15.12 other = $45.35 total per patient. (2) Bradley et al. 2021 CEA of solar-powered O2: $26/patient treated (JAMA Network Open, PMID 34165579). (3) Lancet Commission 2025: $59/DALY averted median (range $21-225), implying higher per-patient costs when accounting for full system costs. Using $45 as best guess: consistent with the original total cost estimate and above the modeled $26 (which may understate real-world implementation costs). If government co-funding is available, philanthropic share would be lower.</t>
       </text>
     </comment>
     <comment ref="C15" authorId="0" shapeId="0">
@@ -197,6 +197,16 @@
     <comment ref="C23" authorId="0" shapeId="0">
       <text>
         <t>Uganda RCT: IRR for neonatal deaths was 1.11 (0.76-1.62, NS). Graham et al. 2019 (Nigeria): aOR for neonates 1.12 (0.56-2.26, NS). Duke et al. 2021 (PNG): IRR 1.11 (0.76-1.62, NS). Neonatal hypoxemia may require CPAP or surfactant rather than simple O2.</t>
+      </text>
+    </comment>
+    <comment ref="C33" authorId="0" shapeId="0">
+      <text>
+        <t>From GiveWell's 2020 moral weights tool. Age-specific values: Post Neonatal (1mo-1yr) = 100.7, 1 to 4yr = 127.3. Weighted average assuming ~40% post-neonatal, ~60% age 1-4 (approximate age distribution of under-5 pneumonia deaths excluding neonates): 0.40 x 100.7 + 0.60 x 127.3 = 116.7, rounded to 117.</t>
+      </text>
+    </comment>
+    <comment ref="C34" authorId="0" shapeId="0">
+      <text>
+        <t>From GiveWell's 2020 moral weights tool. Adult oxygen patients include maternal, surgical, and respiratory cases. Assumed age distribution centered on 25-40: 20-24yr=118, 25-29yr=112.7, 30-34yr=106.3, 35-39yr=99.7, 40-44yr=86.4, 45-49yr=75.7. Weighted average ~100. This is still an assumption about age mix — adult contribution is small (~2% of total UoV) so imprecision here matters little.</t>
       </text>
     </comment>
     <comment ref="C37" authorId="0" shapeId="0">
@@ -536,15 +546,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Cost per patient receiving oxygen (philanthropic)</t>
+          <t>Cost per patient receiving oxygen (total program cost)</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Mid-range: CHAI costs ~$15/patient; total with government match ~$45</t>
+          <t>Total cost per patient including infrastructure, training, and consumables</t>
         </is>
       </c>
     </row>
@@ -903,15 +913,15 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Moral weight per under-5 death averted (UoV)</t>
+          <t>Moral weight per child (1mo-5yr) death averted (UoV)</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>GiveWell standard</t>
+        <v>117</v>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>GiveWell 2020 moral weights: Post Neonatal 100.7, 1-4yr 127.3</t>
         </is>
       </c>
     </row>
@@ -922,11 +932,11 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>30</v>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>Rough estimate; average age ~35-50, mix of surgical/maternal</t>
+        <v>100</v>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>GiveWell 2020 moral weights: weighted avg across ages 20-50</t>
         </is>
       </c>
     </row>
@@ -1047,63 +1057,63 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CE at $15/patient</t>
+          <t>CE at $26/patient</t>
         </is>
       </c>
       <c r="B45" s="13">
-        <f>((B2/15*B7*B8*B15*(1-B16)*B17*B18*B33)+(B2/15*B7*B10*B26*(1-B27)*B28*B34))*(1+B37)/(B2*B41)</f>
+        <f>((B2/26*B7*B8*B15*(1-B16)*B17*B18*B33)+(B2/26*B7*B10*B26*(1-B27)*B28*B34))*(1+B37)/(B2*B41)</f>
         <v/>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Scenario: CHAI-only cost, no overhead</t>
+          <t>Scenario: Bradley et al. 2021 modeled cost for solar O2 systems</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CE at $20/patient</t>
+          <t>CE at $45/patient (best guess)</t>
         </is>
       </c>
       <c r="B46" s="13">
-        <f>((B2/20*B7*B8*B15*(1-B16)*B17*B18*B33)+(B2/20*B7*B10*B26*(1-B27)*B28*B34))*(1+B37)/(B2*B41)</f>
-        <v/>
-      </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>Scenario: lean implementation</t>
-        </is>
+        <f>B42</f>
+        <v/>
+      </c>
+      <c r="C46" s="5">
+        <f> main BOTEC estimate</f>
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CE at $30/patient (best guess)</t>
+          <t>CE at $75/patient</t>
         </is>
       </c>
       <c r="B47" s="13">
-        <f>B42</f>
-        <v/>
-      </c>
-      <c r="C47" s="5">
-        <f> main BOTEC estimate</f>
-        <v/>
+        <f>((B2/75*B7*B8*B15*(1-B16)*B17*B18*B33)+(B2/75*B7*B10*B26*(1-B27)*B28*B34))*(1+B37)/(B2*B41)</f>
+        <v/>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Scenario: high-cost implementation with solar + remote facilities</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CE at $50/patient</t>
+          <t>CE at $100/patient</t>
         </is>
       </c>
       <c r="B48" s="13">
-        <f>((B2/50*B7*B8*B15*(1-B16)*B17*B18*B33)+(B2/50*B7*B10*B26*(1-B27)*B28*B34))*(1+B37)/(B2*B41)</f>
+        <f>((B2/100*B7*B8*B15*(1-B16)*B17*B18*B33)+(B2/100*B7*B10*B26*(1-B27)*B28*B34))*(1+B37)/(B2*B41)</f>
         <v/>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Scenario: high-cost rural solar-powered systems</t>
+          <t>Scenario: pessimistic — full system costs in difficult settings</t>
         </is>
       </c>
     </row>
@@ -1111,6 +1121,8 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>